<commit_message>
generated week 5 queries, commit (2/2).
</commit_message>
<xml_diff>
--- a/Function 6/evals.xlsx
+++ b/Function 6/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1E96F6-EEB2-4071-8B66-2C844B75A131}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5ECA01B-0CC4-4521-8258-D5205D23439D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -529,7 +529,9 @@
         <v>0.13104946794814401</v>
       </c>
       <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
+      <c r="N6" s="2">
+        <v>-0.51212104765767597</v>
+      </c>
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
@@ -537,15 +539,25 @@
         <v>5</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2">
+        <v>0.48706930601068998</v>
+      </c>
       <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="F7" s="2">
+        <v>0.27966911407105199</v>
+      </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2">
+        <v>0.61445146217359103</v>
+      </c>
       <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+      <c r="J7" s="2">
+        <v>0.67727561258672297</v>
+      </c>
       <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
+      <c r="L7" s="2">
+        <v>4.8755396867951099E-2</v>
+      </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -650,12 +662,58 @@
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
     <mergeCell ref="N5:O5"/>
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="L5:M5"/>
@@ -668,58 +726,12 @@
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="N4:O4"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="N7:O7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
generated week 7 queries (2/2).
</commit_message>
<xml_diff>
--- a/Function 6/evals.xlsx
+++ b/Function 6/evals.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E798E6-3926-43E0-9CA8-7610EF07367A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EAA8E62-091D-4970-8EDB-EB78B18A0678}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -382,9 +382,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:O14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -414,7 +414,7 @@
       </c>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B3" s="3">
         <v>1</v>
       </c>
@@ -444,7 +444,7 @@
       </c>
       <c r="O3" s="2"/>
     </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B4" s="3">
         <v>2</v>
       </c>
@@ -474,7 +474,7 @@
       </c>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B5" s="3">
         <v>3</v>
       </c>
@@ -504,7 +504,7 @@
       </c>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B6" s="3">
         <v>4</v>
       </c>
@@ -534,7 +534,7 @@
       </c>
       <c r="O6" s="2"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="3">
         <v>5</v>
       </c>
@@ -564,7 +564,7 @@
       </c>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
         <v>6</v>
       </c>
@@ -594,7 +594,7 @@
       </c>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>7</v>
       </c>
@@ -619,26 +619,44 @@
         <v>0</v>
       </c>
       <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
+      <c r="N9" s="2">
+        <v>-0.50358841113939301</v>
+      </c>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B10" s="3">
+        <v>8</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="2">
+        <v>0.47964295799669698</v>
+      </c>
       <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2">
+        <v>0.32659767809933599</v>
+      </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2">
+        <v>0.58735135524740201</v>
+      </c>
       <c r="I10" s="2"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
+      <c r="J10" s="2">
+        <v>0.75390768544999098</v>
+      </c>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2">
+        <v>0.18075518442504199</v>
+      </c>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B11" s="3">
+        <v>9</v>
+      </c>
+      <c r="C11" s="3"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -650,7 +668,7 @@
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -664,7 +682,7 @@
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -678,7 +696,7 @@
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -693,19 +711,62 @@
       <c r="M14" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="76">
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="N8:O8"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="N7:O7"/>
+  <mergeCells count="79">
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
     <mergeCell ref="N5:O5"/>
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="L5:M5"/>
@@ -718,58 +779,18 @@
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="N4:O4"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="N9:O9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
week 10 queries generated (2/2).
</commit_message>
<xml_diff>
--- a/Function 6/evals.xlsx
+++ b/Function 6/evals.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C63BC1E-125D-4999-939A-99A092D69E8E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C7FB16-7D2F-4463-A6BE-4DA35DF872F3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -382,9 +382,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:O14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -414,7 +414,7 @@
       </c>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B3" s="3">
         <v>1</v>
       </c>
@@ -444,7 +444,7 @@
       </c>
       <c r="O3" s="2"/>
     </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B4" s="3">
         <v>2</v>
       </c>
@@ -474,7 +474,7 @@
       </c>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B5" s="3">
         <v>3</v>
       </c>
@@ -504,7 +504,7 @@
       </c>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B6" s="3">
         <v>4</v>
       </c>
@@ -534,7 +534,7 @@
       </c>
       <c r="O6" s="2"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="3">
         <v>5</v>
       </c>
@@ -564,7 +564,7 @@
       </c>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
         <v>6</v>
       </c>
@@ -594,7 +594,7 @@
       </c>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>7</v>
       </c>
@@ -624,7 +624,7 @@
       </c>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>8</v>
       </c>
@@ -654,7 +654,7 @@
       </c>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>9</v>
       </c>
@@ -679,28 +679,40 @@
         <v>0.191095323422066</v>
       </c>
       <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
+      <c r="N11" s="2">
+        <v>-0.34514647441403101</v>
+      </c>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <v>10</v>
       </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="2"/>
+      <c r="D12" s="2">
+        <v>0.45738726168011901</v>
+      </c>
       <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="F12" s="2">
+        <v>0.43081774904776599</v>
+      </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
+      <c r="H12" s="2">
+        <v>0.577587755113945</v>
+      </c>
       <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
+      <c r="J12" s="2">
+        <v>0.73080854779929205</v>
+      </c>
       <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
+      <c r="L12" s="2">
+        <v>0.16413369296096</v>
+      </c>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <v>11</v>
       </c>
@@ -718,7 +730,7 @@
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -734,24 +746,64 @@
     </row>
   </sheetData>
   <mergeCells count="88">
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="N8:O8"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
     <mergeCell ref="N5:O5"/>
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="L5:M5"/>
@@ -764,64 +816,24 @@
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="N4:O4"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="J13:K13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
week 11 queries generated (2/2)
</commit_message>
<xml_diff>
--- a/Function 6/evals.xlsx
+++ b/Function 6/evals.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C7FB16-7D2F-4463-A6BE-4DA35DF872F3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F3D43A-B6E0-4BE3-A859-0C4F0DD31824}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -89,9 +89,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -382,386 +381,447 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:O14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B2" s="3" t="s">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="2"/>
+      <c r="F2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="2"/>
+      <c r="H2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3" t="s">
+      <c r="I2" s="2"/>
+      <c r="J2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3" t="s">
+      <c r="K2" s="2"/>
+      <c r="L2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="3" t="s">
+      <c r="M2" s="1"/>
+      <c r="N2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="O2" s="2"/>
-    </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B3" s="3">
+      <c r="O2" s="1"/>
+    </row>
+    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B3" s="2">
         <v>1</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="2">
+      <c r="C3" s="2"/>
+      <c r="D3" s="1">
         <v>0.28513226139336401</v>
       </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2">
+      <c r="E3" s="1"/>
+      <c r="F3" s="1">
         <v>0</v>
       </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="4">
+      <c r="G3" s="1"/>
+      <c r="H3" s="3">
         <v>0.59778317071714704</v>
       </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="2">
+      <c r="I3" s="3"/>
+      <c r="J3" s="1">
         <v>1</v>
       </c>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2">
+      <c r="K3" s="1"/>
+      <c r="L3" s="1">
         <v>0</v>
       </c>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2">
+      <c r="M3" s="1"/>
+      <c r="N3" s="1">
         <v>-0.82197116627998901</v>
       </c>
-      <c r="O3" s="2"/>
-    </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B4" s="3">
+      <c r="O3" s="1"/>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B4" s="2">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="2">
+      <c r="C4" s="2"/>
+      <c r="D4" s="1">
         <v>0.35840106518858</v>
       </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2">
+      <c r="E4" s="1"/>
+      <c r="F4" s="1">
         <v>0</v>
       </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1">
         <v>1</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2">
+      <c r="I4" s="1"/>
+      <c r="J4" s="1">
         <v>1</v>
       </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2">
+      <c r="K4" s="1"/>
+      <c r="L4" s="1">
         <v>1</v>
       </c>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2">
+      <c r="M4" s="1"/>
+      <c r="N4" s="1">
         <v>-1.86163608470941</v>
       </c>
-      <c r="O4" s="2"/>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B5" s="3">
+      <c r="O4" s="1"/>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B5" s="2">
         <v>3</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="2">
+      <c r="C5" s="2"/>
+      <c r="D5" s="1">
         <v>0.307293914419835</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2">
+      <c r="E5" s="1"/>
+      <c r="F5" s="1">
         <v>0.52142198776883497</v>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2">
+      <c r="G5" s="1"/>
+      <c r="H5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2">
+      <c r="I5" s="1"/>
+      <c r="J5" s="1">
         <v>1</v>
       </c>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2">
+      <c r="K5" s="1"/>
+      <c r="L5" s="1">
         <v>0</v>
       </c>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2">
+      <c r="M5" s="1"/>
+      <c r="N5" s="1">
         <v>-1.2538706925373599</v>
       </c>
-      <c r="O5" s="2"/>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B6" s="3">
+      <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B6" s="2">
         <v>4</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="2">
+      <c r="C6" s="2"/>
+      <c r="D6" s="1">
         <v>0.49552104045754902</v>
       </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1">
         <v>0.37287270283526502</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2">
+      <c r="G6" s="1"/>
+      <c r="H6" s="1">
         <v>0.80411021791892101</v>
       </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2">
+      <c r="I6" s="1"/>
+      <c r="J6" s="1">
         <v>1</v>
       </c>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2">
+      <c r="K6" s="1"/>
+      <c r="L6" s="1">
         <v>0.13104946794814401</v>
       </c>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2">
+      <c r="M6" s="1"/>
+      <c r="N6" s="1">
         <v>-0.51212104765767597</v>
       </c>
-      <c r="O6" s="2"/>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B7" s="3">
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B7" s="2">
         <v>5</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="2">
+      <c r="C7" s="2"/>
+      <c r="D7" s="1">
         <v>0.48706930601068998</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2">
+      <c r="E7" s="1"/>
+      <c r="F7" s="1">
         <v>0.27966911407105199</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2">
+      <c r="G7" s="1"/>
+      <c r="H7" s="1">
         <v>0.61445146217359103</v>
       </c>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2">
+      <c r="I7" s="1"/>
+      <c r="J7" s="1">
         <v>0.67727561258672297</v>
       </c>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2">
+      <c r="K7" s="1"/>
+      <c r="L7" s="1">
         <v>4.8755396867951099E-2</v>
       </c>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2">
+      <c r="M7" s="1"/>
+      <c r="N7" s="1">
         <v>-0.35302587644018701</v>
       </c>
-      <c r="O7" s="2"/>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B8" s="3">
+      <c r="O7" s="1"/>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B8" s="2">
         <v>6</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="2">
+      <c r="C8" s="2"/>
+      <c r="D8" s="1">
         <v>0.52720929567840602</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2">
+      <c r="E8" s="1"/>
+      <c r="F8" s="1">
         <v>0.294988024664048</v>
       </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2">
+      <c r="G8" s="1"/>
+      <c r="H8" s="1">
         <v>0.53996646486502298</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2">
+      <c r="I8" s="1"/>
+      <c r="J8" s="1">
         <v>0.84896343696642595</v>
       </c>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2">
+      <c r="K8" s="1"/>
+      <c r="L8" s="1">
         <v>0</v>
       </c>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2">
+      <c r="M8" s="1"/>
+      <c r="N8" s="1">
         <v>-0.44067637326828002</v>
       </c>
-      <c r="O8" s="2"/>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B9" s="3">
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B9" s="2">
         <v>7</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="2">
+      <c r="C9" s="2"/>
+      <c r="D9" s="1">
         <v>0.46761052611480303</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2">
+      <c r="E9" s="1"/>
+      <c r="F9" s="1">
         <v>0.26711323427078698</v>
       </c>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2">
+      <c r="G9" s="1"/>
+      <c r="H9" s="1">
         <v>0.83997925618187796</v>
       </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2">
+      <c r="I9" s="1"/>
+      <c r="J9" s="1">
         <v>0.68828418319584805</v>
       </c>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2">
+      <c r="K9" s="1"/>
+      <c r="L9" s="1">
         <v>0</v>
       </c>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2">
+      <c r="M9" s="1"/>
+      <c r="N9" s="1">
         <v>-0.50358841113939301</v>
       </c>
-      <c r="O9" s="2"/>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B10" s="3">
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B10" s="2">
         <v>8</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="2">
+      <c r="C10" s="2"/>
+      <c r="D10" s="1">
         <v>0.47964295799669698</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1">
         <v>0.32659767809933599</v>
       </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2">
+      <c r="G10" s="1"/>
+      <c r="H10" s="1">
         <v>0.58735135524740201</v>
       </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2">
+      <c r="I10" s="1"/>
+      <c r="J10" s="1">
         <v>0.75390768544999098</v>
       </c>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2">
+      <c r="K10" s="1"/>
+      <c r="L10" s="1">
         <v>0.18075518442504199</v>
       </c>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2">
+      <c r="M10" s="1"/>
+      <c r="N10" s="1">
         <v>-0.272387516817372</v>
       </c>
-      <c r="O10" s="2"/>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B11" s="3">
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B11" s="2">
         <v>9</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="2">
+      <c r="C11" s="2"/>
+      <c r="D11" s="1">
         <v>0.47328871612129902</v>
       </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1">
         <v>0.27383177725598501</v>
       </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2">
+      <c r="G11" s="1"/>
+      <c r="H11" s="1">
         <v>0.59342929576552905</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2">
+      <c r="I11" s="1"/>
+      <c r="J11" s="1">
         <v>0.76203790388685599</v>
       </c>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2">
+      <c r="K11" s="1"/>
+      <c r="L11" s="1">
         <v>0.191095323422066</v>
       </c>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2">
+      <c r="M11" s="1"/>
+      <c r="N11" s="1">
         <v>-0.34514647441403101</v>
       </c>
-      <c r="O11" s="2"/>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B12" s="3">
+      <c r="O11" s="1"/>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B12" s="2">
         <v>10</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="2">
+      <c r="C12" s="2"/>
+      <c r="D12" s="1">
         <v>0.45738726168011901</v>
       </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2">
+      <c r="E12" s="1"/>
+      <c r="F12" s="1">
         <v>0.43081774904776599</v>
       </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2">
+      <c r="G12" s="1"/>
+      <c r="H12" s="1">
         <v>0.577587755113945</v>
       </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2">
+      <c r="I12" s="1"/>
+      <c r="J12" s="1">
         <v>0.73080854779929205</v>
       </c>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2">
+      <c r="K12" s="1"/>
+      <c r="L12" s="1">
         <v>0.16413369296096</v>
       </c>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B13" s="3">
+      <c r="M12" s="1"/>
+      <c r="N12" s="1">
+        <v>-0.31607564629949603</v>
+      </c>
+      <c r="O12" s="1"/>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B13" s="2">
         <v>11</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-    </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="1">
+        <v>0.51181173317557205</v>
+      </c>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1">
+        <v>0.36131515534559899</v>
+      </c>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1">
+        <v>0.60679906312851795</v>
+      </c>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1">
+        <v>0.72484193707247402</v>
+      </c>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1">
+        <v>0.16665263431482699</v>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="88">
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
+  <mergeCells count="91">
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="N5:O5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
@@ -774,66 +834,22 @@
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="N5:O5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="N7:O7"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="N8:O8"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="J11:K11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>